<commit_message>
orden de accesos y aviso de corte
</commit_message>
<xml_diff>
--- a/actualizacion/enlaces.xlsx
+++ b/actualizacion/enlaces.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mi unidad\CH_projects\SDIS\COLJ\tablero-calidad-colj\actualizacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8759A72C-FE3B-4282-A135-B81DBF3B7BB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C20D3A75-8C73-4757-B28A-8BE64ED88239}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="24">
   <si>
     <t>Enlaces del tablero COLJ</t>
   </si>
@@ -83,6 +83,15 @@
   </si>
   <si>
     <t>Gemini Notebook 2026</t>
+  </si>
+  <si>
+    <t>Excel de seguimiento de los COLJ</t>
+  </si>
+  <si>
+    <t>Excel vinculado al forms de los COLJ</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/spreadsheets/d/1IxTTkF4sZgHvKNDGGJX9f1eLetgUrbPtSoYWHoIMD3s/edit?usp=sharing</t>
   </si>
 </sst>
 </file>
@@ -461,7 +470,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -494,67 +503,78 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="B5" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B8" t="s">
         <v>15</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s">
         <v>15</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>18</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B11" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C11" s="3" t="s">
         <v>19</v>
       </c>
     </row>
@@ -563,11 +583,12 @@
     <mergeCell ref="A2:C2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="C5" r:id="rId1" display="https://sdisgovco.sharepoint.com/sites/SubdireccindeJuventudPoliticaPblica/Documentos%20compartidos/Forms/AllItems.aspx?d=w51f1c999a8b54dafb1aba57e1b1c1ef7&amp;csf=1&amp;web=1&amp;e=GnCWLh&amp;or=WORD%2DWEB%2EBODY%2ENT&amp;ct=1787615071953&amp;CID=ab08e4f8%2Db68c%2D4040%2Db7c4%2Dad5f5470a599&amp;FolderCTID=0x012000F3947AFB90C3E34881371E69DC98F757&amp;id=%2Fsites%2FSubdireccindeJuventudPoliticaPblica%2FDocumentos%20compartidos%2FInstancias%20de%20participaci%C3%B3n%2FCOLJ" xr:uid="{9DEC7A09-7042-4940-86EF-791B96B76BED}"/>
-    <hyperlink ref="C6" r:id="rId2" xr:uid="{2119B8F4-AF1D-4FAB-B2B0-6185EDD07DBE}"/>
-    <hyperlink ref="C7" r:id="rId3" xr:uid="{911C624D-5B5C-4BBA-A00C-D527DC92DD54}"/>
-    <hyperlink ref="C8" r:id="rId4" xr:uid="{C87C6B01-CF93-44AA-9EE3-F727F3019002}"/>
-    <hyperlink ref="C10" r:id="rId5" xr:uid="{90B37D02-675E-485A-8A70-67D3E05C2F1C}"/>
+    <hyperlink ref="C6" r:id="rId1" display="https://sdisgovco.sharepoint.com/sites/SubdireccindeJuventudPoliticaPblica/Documentos%20compartidos/Forms/AllItems.aspx?d=w51f1c999a8b54dafb1aba57e1b1c1ef7&amp;csf=1&amp;web=1&amp;e=GnCWLh&amp;or=WORD%2DWEB%2EBODY%2ENT&amp;ct=1787615071953&amp;CID=ab08e4f8%2Db68c%2D4040%2Db7c4%2Dad5f5470a599&amp;FolderCTID=0x012000F3947AFB90C3E34881371E69DC98F757&amp;id=%2Fsites%2FSubdireccindeJuventudPoliticaPblica%2FDocumentos%20compartidos%2FInstancias%20de%20participaci%C3%B3n%2FCOLJ" xr:uid="{9DEC7A09-7042-4940-86EF-791B96B76BED}"/>
+    <hyperlink ref="C7" r:id="rId2" xr:uid="{2119B8F4-AF1D-4FAB-B2B0-6185EDD07DBE}"/>
+    <hyperlink ref="C8" r:id="rId3" xr:uid="{911C624D-5B5C-4BBA-A00C-D527DC92DD54}"/>
+    <hyperlink ref="C9" r:id="rId4" xr:uid="{C87C6B01-CF93-44AA-9EE3-F727F3019002}"/>
+    <hyperlink ref="C11" r:id="rId5" xr:uid="{90B37D02-675E-485A-8A70-67D3E05C2F1C}"/>
+    <hyperlink ref="C5" r:id="rId6" xr:uid="{ED939714-8AE9-46D9-A828-42AEF9E56D37}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Agregar el Decreto 647 a enlaces y destacar el nombre del comité en la portada
</commit_message>
<xml_diff>
--- a/actualizacion/enlaces.xlsx
+++ b/actualizacion/enlaces.xlsx
@@ -76,7 +76,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -85,6 +85,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -451,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="5" min="1" max="1"/>
@@ -473,7 +474,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -610,7 +610,7 @@
         </is>
       </c>
     </row>
-    <row r="12">
+    <row r="12" s="5">
       <c r="A12" t="inlineStr">
         <is>
           <t>Tablero Power BI Hackaton 2025</t>
@@ -624,6 +624,23 @@
       <c r="C12" s="3" t="inlineStr">
         <is>
           <t>https://app.powerbi.com/view?r=eyJrIjoiZjVkMDBlMDUtM2Q3Zi00N2EzLTkwMGEtMjQwMjA5MTkyYjE4IiwidCI6ImIzZTMwODA4LWU5YTgtNGYyYS05YmMxLWE3NjBhZTkxMGNmNSIsImMiOjR9</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Decreto 647 de 2025</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Abre en los artículos de los COLJ (133 a 138): funciones, integrantes, secretaría técnica y sesiones.</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>https://www.alcaldiabogota.gov.co/sisjur/normas/Norma1.jsp?i=191867#133</t>
         </is>
       </c>
     </row>

</xml_diff>